<commit_message>
demo: update mda forms
</commit_message>
<xml_diff>
--- a/Demo/MDA/demo_mda_9999_1_location.xlsx
+++ b/Demo/MDA/demo_mda_9999_1_location.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yumbad\Repositories\dsa-forms\Demo\MDA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bonhe\Repositories\dsa-forms\Demo\MDA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E120B472-3A85-4198-A4FD-B1CB12F32477}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92CCE308-89F7-4F6A-99F1-35A4720D47B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="176">
   <si>
     <t>type</t>
   </si>
@@ -496,12 +496,6 @@
     <t>${l_eligible_boy_0_4} + ${l_eligible_girl_0_4} + ${l_eligible_boy_5_14} + ${l_eligible_girl_5_14} + ${l_eligible_boy_15_more} + ${l_eligible_girl_15_more}</t>
   </si>
   <si>
-    <t>(Demo) 1. MDA Location Form V2</t>
-  </si>
-  <si>
-    <t>demo_mda_9999_1_location_v2</t>
-  </si>
-  <si>
     <t>l_recorder_id</t>
   </si>
   <si>
@@ -548,6 +542,27 @@
   </si>
   <si>
     <t>Select the recorder ID</t>
+  </si>
+  <si>
+    <t>${l_state}</t>
+  </si>
+  <si>
+    <t>demo_mda_9999_1_location_v2_1</t>
+  </si>
+  <si>
+    <t>(Demo) 1. MDA Location Form V2.1</t>
+  </si>
+  <si>
+    <t>${l_district}</t>
+  </si>
+  <si>
+    <t>${l_health_facility}</t>
+  </si>
+  <si>
+    <t>bind::db_add_col_5</t>
+  </si>
+  <si>
+    <t>${l_location}</t>
   </si>
 </sst>
 </file>
@@ -992,7 +1007,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q20"/>
+  <dimension ref="A1:R20"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="28" style="4" bestFit="1" customWidth="1"/>
@@ -1012,10 +1027,11 @@
     <col min="15" max="15" width="18" style="4" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="20.875" style="4" customWidth="1"/>
     <col min="17" max="17" width="20.375" style="4" customWidth="1"/>
-    <col min="18" max="16384" width="11" style="4"/>
+    <col min="18" max="18" width="18" style="4" bestFit="1" customWidth="1"/>
+    <col min="19" max="16384" width="11" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="1" customFormat="1">
+    <row r="1" spans="1:18" s="1" customFormat="1">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -1067,16 +1083,19 @@
       <c r="Q1" s="21" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" s="3" customFormat="1">
+      <c r="R1" s="21" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" s="3" customFormat="1">
       <c r="A2" s="15" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D2" s="22"/>
       <c r="E2" s="15"/>
@@ -1092,8 +1111,9 @@
       <c r="O2" s="23"/>
       <c r="P2" s="23"/>
       <c r="Q2" s="23"/>
-    </row>
-    <row r="3" spans="1:17" ht="26.25">
+      <c r="R2" s="16"/>
+    </row>
+    <row r="3" spans="1:18" ht="26.25">
       <c r="A3" s="9" t="s">
         <v>36</v>
       </c>
@@ -1121,8 +1141,9 @@
       <c r="O3" s="9"/>
       <c r="P3" s="9"/>
       <c r="Q3" s="9"/>
-    </row>
-    <row r="4" spans="1:17" ht="26.25">
+      <c r="R3" s="9"/>
+    </row>
+    <row r="4" spans="1:18" ht="26.25">
       <c r="A4" s="9" t="s">
         <v>37</v>
       </c>
@@ -1146,14 +1167,17 @@
         <v>40</v>
       </c>
       <c r="M4" s="9"/>
-      <c r="N4" s="9"/>
+      <c r="N4" s="9" t="s">
+        <v>169</v>
+      </c>
       <c r="O4" s="13" t="s">
         <v>25</v>
       </c>
       <c r="P4" s="9"/>
       <c r="Q4" s="9"/>
-    </row>
-    <row r="5" spans="1:17" ht="26.25">
+      <c r="R4" s="9"/>
+    </row>
+    <row r="5" spans="1:18" ht="26.25">
       <c r="A5" s="9" t="s">
         <v>131</v>
       </c>
@@ -1178,11 +1202,16 @@
       </c>
       <c r="M5" s="9"/>
       <c r="N5" s="9"/>
-      <c r="O5" s="9"/>
-      <c r="P5" s="13"/>
+      <c r="O5" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="P5" s="13" t="s">
+        <v>25</v>
+      </c>
       <c r="Q5" s="9"/>
-    </row>
-    <row r="6" spans="1:17" ht="33.75">
+      <c r="R5" s="9"/>
+    </row>
+    <row r="6" spans="1:18" ht="33.75">
       <c r="A6" s="9" t="s">
         <v>132</v>
       </c>
@@ -1208,12 +1237,15 @@
       <c r="M6" s="9"/>
       <c r="N6" s="9"/>
       <c r="O6" s="9"/>
-      <c r="P6" s="13" t="s">
+      <c r="P6" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="Q6" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="Q6" s="9"/>
-    </row>
-    <row r="7" spans="1:17" ht="26.25">
+      <c r="R6" s="9"/>
+    </row>
+    <row r="7" spans="1:18" ht="26.25">
       <c r="A7" s="9" t="s">
         <v>133</v>
       </c>
@@ -1240,11 +1272,14 @@
       <c r="N7" s="9"/>
       <c r="O7" s="9"/>
       <c r="P7" s="9"/>
-      <c r="Q7" s="13" t="s">
+      <c r="Q7" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="R7" s="13" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:17">
+    <row r="8" spans="1:18">
       <c r="A8" s="9" t="s">
         <v>47</v>
       </c>
@@ -1270,8 +1305,9 @@
       <c r="O8" s="9"/>
       <c r="P8" s="9"/>
       <c r="Q8" s="9"/>
-    </row>
-    <row r="9" spans="1:17">
+      <c r="R8" s="9"/>
+    </row>
+    <row r="9" spans="1:18">
       <c r="A9" s="9" t="s">
         <v>47</v>
       </c>
@@ -1297,8 +1333,9 @@
       <c r="O9" s="9"/>
       <c r="P9" s="9"/>
       <c r="Q9" s="9"/>
-    </row>
-    <row r="10" spans="1:17">
+      <c r="R9" s="9"/>
+    </row>
+    <row r="10" spans="1:18">
       <c r="A10" s="9" t="s">
         <v>47</v>
       </c>
@@ -1324,8 +1361,9 @@
       <c r="O10" s="9"/>
       <c r="P10" s="9"/>
       <c r="Q10" s="9"/>
-    </row>
-    <row r="11" spans="1:17">
+      <c r="R10" s="9"/>
+    </row>
+    <row r="11" spans="1:18">
       <c r="A11" s="9" t="s">
         <v>47</v>
       </c>
@@ -1351,8 +1389,9 @@
       <c r="O11" s="9"/>
       <c r="P11" s="9"/>
       <c r="Q11" s="9"/>
-    </row>
-    <row r="12" spans="1:17">
+      <c r="R11" s="9"/>
+    </row>
+    <row r="12" spans="1:18">
       <c r="A12" s="9" t="s">
         <v>47</v>
       </c>
@@ -1378,8 +1417,9 @@
       <c r="O12" s="9"/>
       <c r="P12" s="9"/>
       <c r="Q12" s="9"/>
-    </row>
-    <row r="13" spans="1:17">
+      <c r="R12" s="9"/>
+    </row>
+    <row r="13" spans="1:18">
       <c r="A13" s="9" t="s">
         <v>47</v>
       </c>
@@ -1405,8 +1445,9 @@
       <c r="O13" s="9"/>
       <c r="P13" s="9"/>
       <c r="Q13" s="9"/>
-    </row>
-    <row r="14" spans="1:17">
+      <c r="R13" s="9"/>
+    </row>
+    <row r="14" spans="1:18">
       <c r="A14" s="9" t="s">
         <v>47</v>
       </c>
@@ -1432,8 +1473,9 @@
       <c r="O14" s="9"/>
       <c r="P14" s="9"/>
       <c r="Q14" s="9"/>
-    </row>
-    <row r="15" spans="1:17">
+      <c r="R14" s="9"/>
+    </row>
+    <row r="15" spans="1:18">
       <c r="A15" s="9" t="s">
         <v>150</v>
       </c>
@@ -1459,8 +1501,9 @@
       <c r="O15" s="9"/>
       <c r="P15" s="9"/>
       <c r="Q15" s="9"/>
-    </row>
-    <row r="16" spans="1:17">
+      <c r="R15" s="9"/>
+    </row>
+    <row r="16" spans="1:18">
       <c r="A16" s="9" t="s">
         <v>14</v>
       </c>
@@ -1488,8 +1531,9 @@
       <c r="O16" s="9"/>
       <c r="P16" s="9"/>
       <c r="Q16" s="9"/>
-    </row>
-    <row r="17" spans="1:17">
+      <c r="R16" s="9"/>
+    </row>
+    <row r="17" spans="1:18">
       <c r="A17" s="9" t="s">
         <v>13</v>
       </c>
@@ -1515,8 +1559,9 @@
       <c r="O17" s="9"/>
       <c r="P17" s="9"/>
       <c r="Q17" s="9"/>
-    </row>
-    <row r="18" spans="1:17">
+      <c r="R17" s="9"/>
+    </row>
+    <row r="18" spans="1:18">
       <c r="A18" s="9" t="s">
         <v>15</v>
       </c>
@@ -1542,8 +1587,9 @@
       <c r="O18" s="9"/>
       <c r="P18" s="9"/>
       <c r="Q18" s="9"/>
-    </row>
-    <row r="19" spans="1:17">
+      <c r="R18" s="9"/>
+    </row>
+    <row r="19" spans="1:18">
       <c r="A19" s="9" t="s">
         <v>55</v>
       </c>
@@ -1565,8 +1611,9 @@
       <c r="O19" s="9"/>
       <c r="P19" s="9"/>
       <c r="Q19" s="9"/>
-    </row>
-    <row r="20" spans="1:17">
+      <c r="R19" s="9"/>
+    </row>
+    <row r="20" spans="1:18">
       <c r="A20" s="9" t="s">
         <v>56</v>
       </c>
@@ -1588,6 +1635,7 @@
       <c r="O20" s="9"/>
       <c r="P20" s="9"/>
       <c r="Q20" s="9"/>
+      <c r="R20" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1632,13 +1680,13 @@
     </row>
     <row r="2" spans="1:7" s="4" customFormat="1">
       <c r="A2" s="16" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D2" s="9"/>
       <c r="E2" s="9"/>
@@ -1647,13 +1695,13 @@
     </row>
     <row r="3" spans="1:7" s="4" customFormat="1">
       <c r="A3" s="16" t="s">
+        <v>154</v>
+      </c>
+      <c r="B3" s="18" t="s">
         <v>156</v>
       </c>
-      <c r="B3" s="18" t="s">
-        <v>158</v>
-      </c>
       <c r="C3" s="19" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -1662,13 +1710,13 @@
     </row>
     <row r="4" spans="1:7" s="4" customFormat="1">
       <c r="A4" s="16" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -1677,13 +1725,13 @@
     </row>
     <row r="5" spans="1:7" s="4" customFormat="1">
       <c r="A5" s="16" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D5" s="9"/>
       <c r="E5" s="9"/>
@@ -1692,13 +1740,13 @@
     </row>
     <row r="6" spans="1:7" s="4" customFormat="1">
       <c r="A6" s="16" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="9"/>
@@ -1707,13 +1755,13 @@
     </row>
     <row r="7" spans="1:7" s="4" customFormat="1">
       <c r="A7" s="16" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D7" s="9"/>
       <c r="E7" s="9"/>
@@ -1722,13 +1770,13 @@
     </row>
     <row r="8" spans="1:7" s="4" customFormat="1">
       <c r="A8" s="16" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D8" s="9"/>
       <c r="E8" s="9"/>
@@ -1737,13 +1785,13 @@
     </row>
     <row r="9" spans="1:7" s="4" customFormat="1">
       <c r="A9" s="16" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
@@ -1752,13 +1800,13 @@
     </row>
     <row r="10" spans="1:7" s="4" customFormat="1">
       <c r="A10" s="16" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
@@ -1767,13 +1815,13 @@
     </row>
     <row r="11" spans="1:7" s="4" customFormat="1">
       <c r="A11" s="16" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
@@ -1782,13 +1830,13 @@
     </row>
     <row r="12" spans="1:7" s="4" customFormat="1">
       <c r="A12" s="16" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
@@ -1797,13 +1845,13 @@
     </row>
     <row r="13" spans="1:7" s="4" customFormat="1">
       <c r="A13" s="16" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
@@ -1812,7 +1860,7 @@
     </row>
     <row r="14" spans="1:7" s="4" customFormat="1">
       <c r="A14" s="16" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B14" s="16">
         <v>99</v>
@@ -3413,10 +3461,10 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="3" t="s">
-        <v>153</v>
+        <v>171</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>154</v>
+        <v>170</v>
       </c>
       <c r="C2" t="s">
         <v>20</v>

</xml_diff>

<commit_message>
demo: udate MDA forms
</commit_message>
<xml_diff>
--- a/Demo/MDA/demo_mda_9999_1_location.xlsx
+++ b/Demo/MDA/demo_mda_9999_1_location.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bonhe\Repositories\dsa-forms\Demo\MDA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yumbad\Repositories\dsa-forms\Demo\MDA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92CCE308-89F7-4F6A-99F1-35A4720D47B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5095D79-9101-4365-8B77-CB5ADF125D38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="170">
   <si>
     <t>type</t>
   </si>
@@ -451,51 +451,12 @@
     <t>location = ${l_location}</t>
   </si>
   <si>
-    <t>Total number of boys aged 0-4 years eligible for treatment</t>
-  </si>
-  <si>
-    <t>Total number of girls aged 0-4 years eligible for treatment</t>
-  </si>
-  <si>
-    <t>Total number of boys aged 5-14 years eligible for treatment</t>
-  </si>
-  <si>
-    <t>Total number of girls aged 5-14 years eligible for treatment</t>
-  </si>
-  <si>
-    <t>Total number of boys aged more than 15 years eligible for treatment</t>
-  </si>
-  <si>
-    <t>Total number of girls aged more than years eligible for treatment</t>
-  </si>
-  <si>
-    <t>l_eligible_boy_0_4</t>
-  </si>
-  <si>
-    <t>l_eligible_boy_5_14</t>
-  </si>
-  <si>
-    <t>l_eligible_girl_0_4</t>
-  </si>
-  <si>
-    <t>l_eligible_girl_5_14</t>
-  </si>
-  <si>
-    <t>l_eligible_boy_15_more</t>
-  </si>
-  <si>
-    <t>l_eligible_girl_15_more</t>
-  </si>
-  <si>
     <t>calculate</t>
   </si>
   <si>
     <t>Total eligible population of the village</t>
   </si>
   <si>
-    <t>${l_eligible_boy_0_4} + ${l_eligible_girl_0_4} + ${l_eligible_boy_5_14} + ${l_eligible_girl_5_14} + ${l_eligible_boy_15_more} + ${l_eligible_girl_15_more}</t>
-  </si>
-  <si>
     <t>l_recorder_id</t>
   </si>
   <si>
@@ -547,12 +508,6 @@
     <t>${l_state}</t>
   </si>
   <si>
-    <t>demo_mda_9999_1_location_v2_1</t>
-  </si>
-  <si>
-    <t>(Demo) 1. MDA Location Form V2.1</t>
-  </si>
-  <si>
     <t>${l_district}</t>
   </si>
   <si>
@@ -563,13 +518,40 @@
   </si>
   <si>
     <t>${l_location}</t>
+  </si>
+  <si>
+    <t>Total number of people aged 15 years and above in the village</t>
+  </si>
+  <si>
+    <t>Total number of people aged 5-14 years of the Village</t>
+  </si>
+  <si>
+    <t>Total number of people aged 1-4 years of the village</t>
+  </si>
+  <si>
+    <t>I_total_popn_1_4</t>
+  </si>
+  <si>
+    <t>I_total_popn_5_14</t>
+  </si>
+  <si>
+    <t>I_total_popn_15_More</t>
+  </si>
+  <si>
+    <t>${I_total_popn_1_4} + ${I_total_popn_5_14} + ${I_total_popn_15_More}</t>
+  </si>
+  <si>
+    <t>(Demo) 1. MDA Location Form V3</t>
+  </si>
+  <si>
+    <t>demo_mda_9999_1_location_v3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -627,6 +609,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -670,7 +659,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -725,6 +714,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1007,7 +999,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R20"/>
+  <dimension ref="A1:R17"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="28" style="4" bestFit="1" customWidth="1"/>
@@ -1084,18 +1076,18 @@
         <v>24</v>
       </c>
       <c r="R1" s="21" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
     </row>
     <row r="2" spans="1:18" s="3" customFormat="1">
       <c r="A2" s="15" t="s">
-        <v>167</v>
+        <v>154</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>153</v>
+        <v>140</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>168</v>
+        <v>155</v>
       </c>
       <c r="D2" s="22"/>
       <c r="E2" s="15"/>
@@ -1168,7 +1160,7 @@
       </c>
       <c r="M4" s="9"/>
       <c r="N4" s="9" t="s">
-        <v>169</v>
+        <v>156</v>
       </c>
       <c r="O4" s="13" t="s">
         <v>25</v>
@@ -1203,7 +1195,7 @@
       <c r="M5" s="9"/>
       <c r="N5" s="9"/>
       <c r="O5" s="9" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="P5" s="13" t="s">
         <v>25</v>
@@ -1238,7 +1230,7 @@
       <c r="N6" s="9"/>
       <c r="O6" s="9"/>
       <c r="P6" s="9" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
       <c r="Q6" s="13" t="s">
         <v>25</v>
@@ -1273,7 +1265,7 @@
       <c r="O7" s="9"/>
       <c r="P7" s="9"/>
       <c r="Q7" s="9" t="s">
-        <v>175</v>
+        <v>160</v>
       </c>
       <c r="R7" s="13" t="s">
         <v>25</v>
@@ -1307,109 +1299,109 @@
       <c r="Q8" s="9"/>
       <c r="R8" s="9"/>
     </row>
-    <row r="9" spans="1:18">
-      <c r="A9" s="9" t="s">
+    <row r="9" spans="1:18" s="26" customFormat="1">
+      <c r="A9" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="B9" s="9" t="s">
-        <v>144</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>138</v>
-      </c>
-      <c r="D9" s="12"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9" t="s">
+      <c r="B9" s="25" t="s">
+        <v>164</v>
+      </c>
+      <c r="C9" s="24" t="s">
+        <v>163</v>
+      </c>
+      <c r="D9" s="24"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="24"/>
+      <c r="H9" s="25"/>
+      <c r="I9" s="25"/>
+      <c r="J9" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="K9" s="9"/>
-      <c r="L9" s="9"/>
-      <c r="M9" s="9"/>
-      <c r="N9" s="9"/>
-      <c r="O9" s="9"/>
-      <c r="P9" s="9"/>
-      <c r="Q9" s="9"/>
-      <c r="R9" s="9"/>
-    </row>
-    <row r="10" spans="1:18">
-      <c r="A10" s="9" t="s">
+      <c r="K9" s="25"/>
+      <c r="L9" s="25"/>
+      <c r="M9" s="25"/>
+      <c r="N9" s="25"/>
+      <c r="O9" s="25"/>
+      <c r="P9" s="25"/>
+      <c r="Q9" s="25"/>
+      <c r="R9" s="25"/>
+    </row>
+    <row r="10" spans="1:18" s="26" customFormat="1">
+      <c r="A10" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="B10" s="9" t="s">
-        <v>146</v>
-      </c>
-      <c r="C10" s="12" t="s">
-        <v>139</v>
-      </c>
-      <c r="D10" s="12"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="12"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9" t="s">
+      <c r="B10" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="C10" s="24" t="s">
+        <v>162</v>
+      </c>
+      <c r="D10" s="24"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="25"/>
+      <c r="I10" s="25"/>
+      <c r="J10" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="K10" s="9"/>
-      <c r="L10" s="9"/>
-      <c r="M10" s="9"/>
-      <c r="N10" s="9"/>
-      <c r="O10" s="9"/>
-      <c r="P10" s="9"/>
-      <c r="Q10" s="9"/>
-      <c r="R10" s="9"/>
-    </row>
-    <row r="11" spans="1:18">
-      <c r="A11" s="9" t="s">
+      <c r="K10" s="25"/>
+      <c r="L10" s="25"/>
+      <c r="M10" s="25"/>
+      <c r="N10" s="25"/>
+      <c r="O10" s="25"/>
+      <c r="P10" s="25"/>
+      <c r="Q10" s="25"/>
+      <c r="R10" s="25"/>
+    </row>
+    <row r="11" spans="1:18" s="26" customFormat="1">
+      <c r="A11" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="B11" s="9" t="s">
-        <v>145</v>
-      </c>
-      <c r="C11" s="12" t="s">
-        <v>140</v>
-      </c>
-      <c r="D11" s="12"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9" t="s">
+      <c r="B11" s="25" t="s">
+        <v>166</v>
+      </c>
+      <c r="C11" s="24" t="s">
+        <v>161</v>
+      </c>
+      <c r="D11" s="24"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="24"/>
+      <c r="H11" s="25"/>
+      <c r="I11" s="25"/>
+      <c r="J11" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="K11" s="9"/>
-      <c r="L11" s="9"/>
-      <c r="M11" s="9"/>
-      <c r="N11" s="9"/>
-      <c r="O11" s="9"/>
-      <c r="P11" s="9"/>
-      <c r="Q11" s="9"/>
-      <c r="R11" s="9"/>
+      <c r="K11" s="25"/>
+      <c r="L11" s="25"/>
+      <c r="M11" s="25"/>
+      <c r="N11" s="25"/>
+      <c r="O11" s="25"/>
+      <c r="P11" s="25"/>
+      <c r="Q11" s="25"/>
+      <c r="R11" s="25"/>
     </row>
     <row r="12" spans="1:18">
       <c r="A12" s="9" t="s">
-        <v>47</v>
+        <v>138</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>147</v>
+        <v>49</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="9"/>
       <c r="F12" s="9"/>
       <c r="G12" s="12"/>
       <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9" t="s">
-        <v>12</v>
-      </c>
+      <c r="I12" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="J12" s="9"/>
       <c r="K12" s="9"/>
       <c r="L12" s="9"/>
       <c r="M12" s="9"/>
@@ -1421,16 +1413,18 @@
     </row>
     <row r="13" spans="1:18">
       <c r="A13" s="9" t="s">
-        <v>47</v>
+        <v>14</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>148</v>
+        <v>50</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>142</v>
+        <v>29</v>
       </c>
       <c r="D13" s="12"/>
-      <c r="E13" s="9"/>
+      <c r="E13" s="9" t="s">
+        <v>51</v>
+      </c>
       <c r="F13" s="9"/>
       <c r="G13" s="12"/>
       <c r="H13" s="9"/>
@@ -1449,13 +1443,13 @@
     </row>
     <row r="14" spans="1:18">
       <c r="A14" s="9" t="s">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>149</v>
+        <v>52</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>143</v>
+        <v>30</v>
       </c>
       <c r="D14" s="12"/>
       <c r="E14" s="9"/>
@@ -1477,23 +1471,23 @@
     </row>
     <row r="15" spans="1:18">
       <c r="A15" s="9" t="s">
-        <v>150</v>
+        <v>15</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>151</v>
+        <v>31</v>
       </c>
       <c r="D15" s="12"/>
       <c r="E15" s="9"/>
       <c r="F15" s="9"/>
       <c r="G15" s="12"/>
       <c r="H15" s="9"/>
-      <c r="I15" s="9" t="s">
-        <v>152</v>
-      </c>
-      <c r="J15" s="9"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="9" t="s">
+        <v>54</v>
+      </c>
       <c r="K15" s="9"/>
       <c r="L15" s="9"/>
       <c r="M15" s="9"/>
@@ -1505,25 +1499,19 @@
     </row>
     <row r="16" spans="1:18">
       <c r="A16" s="9" t="s">
-        <v>14</v>
+        <v>55</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>29</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="C16" s="12"/>
       <c r="D16" s="12"/>
-      <c r="E16" s="9" t="s">
-        <v>51</v>
-      </c>
+      <c r="E16" s="9"/>
       <c r="F16" s="9"/>
       <c r="G16" s="12"/>
       <c r="H16" s="9"/>
       <c r="I16" s="9"/>
-      <c r="J16" s="9" t="s">
-        <v>12</v>
-      </c>
+      <c r="J16" s="9"/>
       <c r="K16" s="9"/>
       <c r="L16" s="9"/>
       <c r="M16" s="9"/>
@@ -1535,23 +1523,19 @@
     </row>
     <row r="17" spans="1:18">
       <c r="A17" s="9" t="s">
-        <v>13</v>
+        <v>56</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>30</v>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="C17" s="12"/>
       <c r="D17" s="12"/>
       <c r="E17" s="9"/>
       <c r="F17" s="9"/>
       <c r="G17" s="12"/>
       <c r="H17" s="9"/>
       <c r="I17" s="9"/>
-      <c r="J17" s="9" t="s">
-        <v>12</v>
-      </c>
+      <c r="J17" s="9"/>
       <c r="K17" s="9"/>
       <c r="L17" s="9"/>
       <c r="M17" s="9"/>
@@ -1561,83 +1545,8 @@
       <c r="Q17" s="9"/>
       <c r="R17" s="9"/>
     </row>
-    <row r="18" spans="1:18">
-      <c r="A18" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B18" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="C18" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="D18" s="12"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="9"/>
-      <c r="I18" s="9"/>
-      <c r="J18" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="K18" s="9"/>
-      <c r="L18" s="9"/>
-      <c r="M18" s="9"/>
-      <c r="N18" s="9"/>
-      <c r="O18" s="9"/>
-      <c r="P18" s="9"/>
-      <c r="Q18" s="9"/>
-      <c r="R18" s="9"/>
-    </row>
-    <row r="19" spans="1:18">
-      <c r="A19" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="B19" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="9"/>
-      <c r="J19" s="9"/>
-      <c r="K19" s="9"/>
-      <c r="L19" s="9"/>
-      <c r="M19" s="9"/>
-      <c r="N19" s="9"/>
-      <c r="O19" s="9"/>
-      <c r="P19" s="9"/>
-      <c r="Q19" s="9"/>
-      <c r="R19" s="9"/>
-    </row>
-    <row r="20" spans="1:18">
-      <c r="A20" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="B20" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="9"/>
-      <c r="I20" s="9"/>
-      <c r="J20" s="9"/>
-      <c r="K20" s="9"/>
-      <c r="L20" s="9"/>
-      <c r="M20" s="9"/>
-      <c r="N20" s="9"/>
-      <c r="O20" s="9"/>
-      <c r="P20" s="9"/>
-      <c r="Q20" s="9"/>
-      <c r="R20" s="9"/>
-    </row>
   </sheetData>
+  <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
@@ -1680,13 +1589,13 @@
     </row>
     <row r="2" spans="1:7" s="4" customFormat="1">
       <c r="A2" s="16" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>155</v>
+        <v>142</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>155</v>
+        <v>142</v>
       </c>
       <c r="D2" s="9"/>
       <c r="E2" s="9"/>
@@ -1695,13 +1604,13 @@
     </row>
     <row r="3" spans="1:7" s="4" customFormat="1">
       <c r="A3" s="16" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>156</v>
+        <v>143</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>156</v>
+        <v>143</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -1710,13 +1619,13 @@
     </row>
     <row r="4" spans="1:7" s="4" customFormat="1">
       <c r="A4" s="16" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>157</v>
+        <v>144</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>157</v>
+        <v>144</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -1725,13 +1634,13 @@
     </row>
     <row r="5" spans="1:7" s="4" customFormat="1">
       <c r="A5" s="16" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>158</v>
+        <v>145</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>158</v>
+        <v>145</v>
       </c>
       <c r="D5" s="9"/>
       <c r="E5" s="9"/>
@@ -1740,13 +1649,13 @@
     </row>
     <row r="6" spans="1:7" s="4" customFormat="1">
       <c r="A6" s="16" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>159</v>
+        <v>146</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>159</v>
+        <v>146</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="9"/>
@@ -1755,13 +1664,13 @@
     </row>
     <row r="7" spans="1:7" s="4" customFormat="1">
       <c r="A7" s="16" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>160</v>
+        <v>147</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>160</v>
+        <v>147</v>
       </c>
       <c r="D7" s="9"/>
       <c r="E7" s="9"/>
@@ -1770,13 +1679,13 @@
     </row>
     <row r="8" spans="1:7" s="4" customFormat="1">
       <c r="A8" s="16" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>161</v>
+        <v>148</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>161</v>
+        <v>148</v>
       </c>
       <c r="D8" s="9"/>
       <c r="E8" s="9"/>
@@ -1785,13 +1694,13 @@
     </row>
     <row r="9" spans="1:7" s="4" customFormat="1">
       <c r="A9" s="16" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>162</v>
+        <v>149</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>162</v>
+        <v>149</v>
       </c>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
@@ -1800,13 +1709,13 @@
     </row>
     <row r="10" spans="1:7" s="4" customFormat="1">
       <c r="A10" s="16" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>163</v>
+        <v>150</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>163</v>
+        <v>150</v>
       </c>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
@@ -1815,13 +1724,13 @@
     </row>
     <row r="11" spans="1:7" s="4" customFormat="1">
       <c r="A11" s="16" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>164</v>
+        <v>151</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>164</v>
+        <v>151</v>
       </c>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
@@ -1830,13 +1739,13 @@
     </row>
     <row r="12" spans="1:7" s="4" customFormat="1">
       <c r="A12" s="16" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>165</v>
+        <v>152</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>165</v>
+        <v>152</v>
       </c>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
@@ -1845,13 +1754,13 @@
     </row>
     <row r="13" spans="1:7" s="4" customFormat="1">
       <c r="A13" s="16" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>166</v>
+        <v>153</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>166</v>
+        <v>153</v>
       </c>
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
@@ -1860,7 +1769,7 @@
     </row>
     <row r="14" spans="1:7" s="4" customFormat="1">
       <c r="A14" s="16" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="B14" s="16">
         <v>99</v>
@@ -3461,10 +3370,10 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="3" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C2" t="s">
         <v>20</v>

</xml_diff>

<commit_message>
wip: update demo forms
</commit_message>
<xml_diff>
--- a/Demo/MDA/demo_mda_9999_1_location.xlsx
+++ b/Demo/MDA/demo_mda_9999_1_location.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yumbad\Repositories\dsa-forms\Demo\MDA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5095D79-9101-4365-8B77-CB5ADF125D38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AA73ED3-59E7-42DD-AC8C-A219E64B33DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>

</xml_diff>